<commit_message>
feat: harden mobile infographic craft and P18 evidence
</commit_message>
<xml_diff>
--- a/examples/p18-synthetic-output-pack/renders/final/recalculated/synthetic-cash-timing-model.xlsx
+++ b/examples/p18-synthetic-output-pack/renders/final/recalculated/synthetic-cash-timing-model.xlsx
@@ -626,11 +626,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="70369630"/>
-        <c:axId val="5003864"/>
+        <c:axId val="53712397"/>
+        <c:axId val="31162063"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="70369630"/>
+        <c:axId val="53712397"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -696,7 +696,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="5003864"/>
+        <c:crossAx val="31162063"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -704,7 +704,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="5003864"/>
+        <c:axId val="31162063"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="50"/>
@@ -782,7 +782,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="70369630"/>
+        <c:crossAx val="53712397"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
         <c:majorUnit val="10"/>

</xml_diff>